<commit_message>
update: atualizacao dos dados de 2024 para 2025
</commit_message>
<xml_diff>
--- a/base_datas/crescimento_medio_populacao_porte.xlsx
+++ b/base_datas/crescimento_medio_populacao_porte.xlsx
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>14.93940593640054</v>
+        <v>15.04874118696193</v>
       </c>
     </row>
     <row r="3">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>45.64195267051103</v>
+        <v>47.18882109496297</v>
       </c>
     </row>
     <row r="4">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>26.02207189185002</v>
+        <v>26.7224480740601</v>
       </c>
     </row>
     <row r="5">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>46.43435162107077</v>
+        <v>47.62649807685909</v>
       </c>
     </row>
     <row r="6">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>9.202743268028778</v>
+        <v>9.573897311441295</v>
       </c>
     </row>
     <row r="7">
@@ -423,7 +423,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>39.72650515740994</v>
+        <v>40.67367932179771</v>
       </c>
     </row>
     <row r="8">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>25.21681644644041</v>
+        <v>25.79284000296109</v>
       </c>
     </row>
     <row r="9">
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>1.891699586481162</v>
+        <v>1.729731992249171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>